<commit_message>
Add highlighted parameter calculation
</commit_message>
<xml_diff>
--- a/six_screenshot_parameter_results.xlsx
+++ b/six_screenshot_parameter_results.xlsx
@@ -998,7 +998,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB7"/>
   <sheetFormatPr defaultRowHeight="14" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1365,6 +1365,83 @@
       </c>
       <c r="AB4" s="7">
         <v>6.1256557731305793E-16</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>128</v>
+      </c>
+      <c r="B7" s="4">
+        <v>256</v>
+      </c>
+      <c r="C7" s="5">
+        <v>15361</v>
+      </c>
+      <c r="D7" s="5">
+        <v>3</v>
+      </c>
+      <c r="E7" s="5">
+        <v>3</v>
+      </c>
+      <c r="F7" s="6">
+        <v>0.81</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0.81</v>
+      </c>
+      <c r="H7" s="5">
+        <v>512</v>
+      </c>
+      <c r="I7" s="5">
+        <v>8</v>
+      </c>
+      <c r="J7" s="7">
+        <v>5.5</v>
+      </c>
+      <c r="K7" s="8">
+        <v>136.57949415623656</v>
+      </c>
+      <c r="L7" s="8">
+        <v>205.56799999999998</v>
+      </c>
+      <c r="M7" s="8">
+        <v>167.024</v>
+      </c>
+      <c r="N7" s="9">
+        <v>1072</v>
+      </c>
+      <c r="O7" s="9">
+        <v>1126</v>
+      </c>
+      <c r="P7" s="9">
+        <v>2198</v>
+      </c>
+      <c r="Q7" s="7">
+        <v>677.8102011625379</v>
+      </c>
+      <c r="R7" s="7">
+        <v>322</v>
+      </c>
+      <c r="S7" s="7">
+        <v>25</v>
+      </c>
+      <c r="T7" s="7">
+        <v>9</v>
+      </c>
+      <c r="U7" s="4">
+        <v>1885</v>
+      </c>
+      <c r="V7" s="7">
+        <v>38081196.97363208</v>
+      </c>
+      <c r="W7" s="10">
+        <v>3796329525551.78</v>
+      </c>
+      <c r="X7" s="7">
+        <v>7072.834956063468</v>
+      </c>
+      <c r="Y7" s="7">
+        <v>7072.834956063468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>